<commit_message>
Correct 1818E Genesis list price to $2,925
Confirmed by Sheffield Pottery; the source sheet printed $2,425, which
was out of line with the $150 Genesis upgrade every other model in the
section carries. Applied through an explicit OVERRIDES table so the
correction is traceable rather than silently baked into the data.

The source's distributor price for that combination ($1,455, i.e. 40%
off the old list) is left as printed and flagged on the Notes sheet.

Also tightens the distributor-price consistency check to the exact
40%/30% discounts the source uses instead of a loose band, which
surfaced a further slip on GF5E / KilnStar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XxJvecb9EHw919ig8p38oT
</commit_message>
<xml_diff>
--- a/Olympic_Kilns_2026_Pricelist.xlsx
+++ b/Olympic_Kilns_2026_Pricelist.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1637" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="646">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -1875,7 +1875,10 @@
     <t xml:space="preserve">Olympic Kilns — 2026 Pricing (effective OCT 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: 2026_New_Pricing_OCT26.xlsx, sheet "Sheet1" — all prices copied from that file, none calculated.</t>
+    <t xml:space="preserve">Source: 2026_New_Pricing_OCT26.xlsx, sheet "Sheet1". Prices are copied from that file, not calculated,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">except for the corrections listed below.</t>
   </si>
   <si>
     <t xml:space="preserve">Olympic Kilns, PO Box 1347, 4225 Thurmon Tanner Pkwy., Flowery Branch, GA 30542 — Sales (800) 241-4400 — olympickilns.com</t>
@@ -1908,31 +1911,49 @@
     <t xml:space="preserve">30% off), shown the same way: a base distributor price plus the distributor cost of each upgrade.</t>
   </si>
   <si>
+    <t xml:space="preserve">Corrections applied to the source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 1818E / Genesis list price set to $2,925 as confirmed by Sheffield Pottery; the source sheet printed $2,425, which was out of line with the $150 Genesis upgrade every other model carries.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source figures that look wrong but were left as printed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• GF5E / KilnStar: distributor $3,240 is 72.0% of list $4,500; the usual 40% off would be $2,700 (source row 331)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• GF17E / Genesis: distributor $11,935 is 87.1% of list $13,700; the usual 30% off would be $9,590 (source row 595)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• GF17E CS / KilnStar: distributor $9,485 is 64.1% of list $14,800; the usual 30% off would be $10,360 (source row 594)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• GF17E CS / Genesis: distributor $25,550 is 170.9% of list $14,950; the usual 30% off would be $10,465 (source row 595)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Carried over from the source as printed</t>
   </si>
   <si>
-    <t xml:space="preserve">• GF17E / Genesis: distributor $11,935 is 87% of list $13,700 (source row 595)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• GF17E CS / Genesis: distributor $25,550 is 171% of list $14,950 (source row 595)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Three models come out with a NEGATIVE upgrade because that is how the source prices them: HB86 Vitrigraph</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  (KilnStar $1,625 vs Spark $1,700), 1818E (Genesis $2,425 vs KilnStar $2,775) and DM2823HE (Genesis $5,835</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  vs KilnStar $5,985). Every other model in those sections adds $125-$150 for Genesis, so 1818E and DM2823HE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  look like typos in the source sheet.</t>
+    <t xml:space="preserve">• 1818E / Genesis distributor price is still the source's $1,455, which was 40% off the old $2,425 list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  40% off the corrected $2,925 list would be $1,755 — confirm with Olympic before quoting dealer cost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  This is why the 1818E row shows a negative Genesis Upgrade D$.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Two models come out with a NEGATIVE upgrade because that is how the source prices them: HB86 Vitrigraph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  (KilnStar $1,625 vs Spark $1,700 — different controllers rather than tiers) and DM2823HE (Genesis $5,835</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  vs KilnStar $5,985, where every other Dual Media model adds $150 for Genesis).</t>
   </si>
   <si>
     <t xml:space="preserve">• 2318HE and GF12E have no distributor price in the source.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• GF17E CS / KilnStar: the source repeats GF17E's distributor price ($9,485); 30% off list would be $10,360.</t>
   </si>
   <si>
     <t xml:space="preserve">• "GE12E CS" is spelled that way in the source (elsewhere GF12E CS).</t>
@@ -4009,7 +4030,7 @@
       </c>
       <c r="F48" s="3" t="n">
         <f aca="false">IF(OR($D48="",INDEX('Controller Prices'!$E:$E,MATCH($B48,'Controller Prices'!$B:$B,0))=""),"",INDEX('Controller Prices'!$E:$E,MATCH($B48,'Controller Prices'!$B:$B,0))-$D48)</f>
-        <v>-350</v>
+        <v>150</v>
       </c>
       <c r="G48" s="3" t="n">
         <v>1665</v>
@@ -10171,7 +10192,7 @@
         <v>2775</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>2425</v>
+        <v>2925</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
@@ -18039,7 +18060,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -18061,15 +18082,15 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7"/>
+      <c r="A4" s="7" t="s">
+        <v>612</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>612</v>
-      </c>
+      <c r="A5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>613</v>
       </c>
     </row>
@@ -18109,15 +18130,15 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7"/>
+      <c r="A14" s="7" t="s">
+        <v>621</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>621</v>
-      </c>
+      <c r="A15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>622</v>
       </c>
     </row>
@@ -18127,81 +18148,122 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="7"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>624</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>625</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>631</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
         <v>632</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>633</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
         <v>638</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>